<commit_message>
Fix bug B02 in calculateDiscount and pass all 6 boundary tests
</commit_message>
<xml_diff>
--- a/Unit_Test_Report.xlsx
+++ b/Unit_Test_Report.xlsx
@@ -2844,7 +2844,7 @@
       <c r="B2" s="139" t="n"/>
       <c r="C2" s="140" t="inlineStr">
         <is>
-          <t>calculateSubtotal</t>
+          <t>calculateSubtotal &amp; calculateDiscount</t>
         </is>
       </c>
       <c r="D2" s="139" t="n"/>
@@ -2861,7 +2861,7 @@
       <c r="K2" s="142" t="n"/>
       <c r="L2" s="143" t="inlineStr">
         <is>
-          <t>Tính thành tiền sản phẩm</t>
+          <t>Tính thành tiền &amp; Chiết khấu</t>
         </is>
       </c>
       <c r="M2" s="139" t="n"/>
@@ -2919,7 +2919,7 @@
       </c>
       <c r="B4" s="146" t="n"/>
       <c r="C4" s="107" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="D4" s="153" t="n"/>
       <c r="E4" s="7" t="n"/>
@@ -2954,7 +2954,7 @@
       <c r="B5" s="146" t="n"/>
       <c r="C5" s="115" t="inlineStr">
         <is>
-          <t>Kiểm thử đơn vị cho phương thức calculateSubtotal(Product product)</t>
+          <t>Kiểm thử đơn vị cho calculateSubtotal &amp; calculateDiscount (6 boundary values)</t>
         </is>
       </c>
       <c r="D5" s="153" t="n"/>
@@ -3019,7 +3019,7 @@
     </row>
     <row r="7" ht="13.5" customHeight="1" thickBot="1">
       <c r="A7" s="162" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="B7" s="163" t="n"/>
       <c r="C7" s="164" t="n">
@@ -3047,7 +3047,7 @@
         <v/>
       </c>
       <c r="O7" s="168" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="P7" s="165" t="n"/>
       <c r="Q7" s="165" t="n"/>
@@ -3088,10 +3088,26 @@
           <t>UTCID05</t>
         </is>
       </c>
-      <c r="K9" s="38" t="n"/>
-      <c r="L9" s="38" t="n"/>
-      <c r="M9" s="38" t="n"/>
-      <c r="N9" s="38" t="n"/>
+      <c r="K9" s="38" t="inlineStr">
+        <is>
+          <t>UTCID06</t>
+        </is>
+      </c>
+      <c r="L9" s="38" t="inlineStr">
+        <is>
+          <t>UTCID07</t>
+        </is>
+      </c>
+      <c r="M9" s="38" t="inlineStr">
+        <is>
+          <t>UTCID08</t>
+        </is>
+      </c>
+      <c r="N9" s="38" t="inlineStr">
+        <is>
+          <t>UTCID09</t>
+        </is>
+      </c>
       <c r="O9" s="38" t="n"/>
       <c r="P9" s="38" t="n"/>
       <c r="Q9" s="38" t="n"/>
@@ -3226,12 +3242,36 @@
           <t>Product = null</t>
         </is>
       </c>
-      <c r="I13" s="11" t="n"/>
-      <c r="J13" s="11" t="n"/>
-      <c r="K13" s="11" t="n"/>
-      <c r="L13" s="11" t="n"/>
-      <c r="M13" s="11" t="n"/>
-      <c r="N13" s="11" t="n"/>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>subtotal = 999.99</t>
+        </is>
+      </c>
+      <c r="J13" s="11" t="inlineStr">
+        <is>
+          <t>subtotal = 1000.0</t>
+        </is>
+      </c>
+      <c r="K13" s="11" t="inlineStr">
+        <is>
+          <t>subtotal = 4999.99</t>
+        </is>
+      </c>
+      <c r="L13" s="11" t="inlineStr">
+        <is>
+          <t>subtotal = 5000.0</t>
+        </is>
+      </c>
+      <c r="M13" s="11" t="inlineStr">
+        <is>
+          <t>subtotal = 9999.99</t>
+        </is>
+      </c>
+      <c r="N13" s="11" t="inlineStr">
+        <is>
+          <t>subtotal = 10000.0</t>
+        </is>
+      </c>
       <c r="O13" s="11" t="n"/>
       <c r="P13" s="11" t="n"/>
       <c r="Q13" s="11" t="n"/>
@@ -3815,12 +3855,36 @@
         </is>
       </c>
       <c r="H38" s="46" t="n"/>
-      <c r="I38" s="46" t="n"/>
-      <c r="J38" s="46" t="n"/>
-      <c r="K38" s="46" t="n"/>
-      <c r="L38" s="46" t="n"/>
-      <c r="M38" s="46" t="n"/>
-      <c r="N38" s="46" t="n"/>
+      <c r="I38" s="46" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="J38" s="46" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="K38" s="46" t="inlineStr">
+        <is>
+          <t>249.9995</t>
+        </is>
+      </c>
+      <c r="L38" s="46" t="inlineStr">
+        <is>
+          <t>500.0</t>
+        </is>
+      </c>
+      <c r="M38" s="46" t="inlineStr">
+        <is>
+          <t>999.999</t>
+        </is>
+      </c>
+      <c r="N38" s="46" t="inlineStr">
+        <is>
+          <t>1500.0</t>
+        </is>
+      </c>
       <c r="O38" s="46" t="n"/>
       <c r="P38" s="46" t="n"/>
       <c r="Q38" s="46" t="n"/>
@@ -4045,12 +4109,36 @@
           <t>A</t>
         </is>
       </c>
-      <c r="I47" s="82" t="n"/>
-      <c r="J47" s="82" t="n"/>
-      <c r="K47" s="82" t="n"/>
-      <c r="L47" s="82" t="n"/>
-      <c r="M47" s="82" t="n"/>
-      <c r="N47" s="82" t="n"/>
+      <c r="I47" s="82" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J47" s="82" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K47" s="82" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="L47" s="82" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="M47" s="82" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="N47" s="82" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="O47" s="82" t="n"/>
       <c r="P47" s="82" t="n"/>
       <c r="Q47" s="82" t="n"/>
@@ -4083,12 +4171,36 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="I48" s="19" t="n"/>
-      <c r="J48" s="19" t="n"/>
-      <c r="K48" s="19" t="n"/>
-      <c r="L48" s="19" t="n"/>
-      <c r="M48" s="19" t="n"/>
-      <c r="N48" s="19" t="n"/>
+      <c r="I48" s="19" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="J48" s="19" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="K48" s="19" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="L48" s="19" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="M48" s="19" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="N48" s="19" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
       <c r="O48" s="19" t="n"/>
       <c r="P48" s="19" t="n"/>
       <c r="Q48" s="19" t="n"/>
@@ -4121,12 +4233,36 @@
           <t>2026-10-04</t>
         </is>
       </c>
-      <c r="I49" s="173" t="n"/>
-      <c r="J49" s="173" t="n"/>
-      <c r="K49" s="173" t="n"/>
-      <c r="L49" s="173" t="n"/>
-      <c r="M49" s="173" t="n"/>
-      <c r="N49" s="173" t="n"/>
+      <c r="I49" s="173" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="J49" s="173" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="K49" s="173" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="L49" s="173" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="M49" s="173" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="N49" s="173" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
       <c r="O49" s="173" t="n"/>
       <c r="P49" s="173" t="n"/>
       <c r="Q49" s="173" t="n"/>
@@ -4159,12 +4295,36 @@
           <t>None</t>
         </is>
       </c>
-      <c r="I50" s="32" t="n"/>
-      <c r="J50" s="32" t="n"/>
-      <c r="K50" s="32" t="n"/>
-      <c r="L50" s="32" t="n"/>
-      <c r="M50" s="32" t="n"/>
-      <c r="N50" s="32" t="n"/>
+      <c r="I50" s="32" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J50" s="32" t="inlineStr">
+        <is>
+          <t>B02 (Fixed)</t>
+        </is>
+      </c>
+      <c r="K50" s="32" t="inlineStr">
+        <is>
+          <t>B02 (Fixed)</t>
+        </is>
+      </c>
+      <c r="L50" s="32" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="M50" s="32" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="N50" s="32" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="O50" s="32" t="n"/>
       <c r="P50" s="32" t="n"/>
       <c r="Q50" s="32" t="n"/>

</xml_diff>

<commit_message>
Add unit tests for calculateShippingFee (Test failing as expected)
</commit_message>
<xml_diff>
--- a/Unit_Test_Report.xlsx
+++ b/Unit_Test_Report.xlsx
@@ -2844,7 +2844,7 @@
       <c r="B2" s="139" t="n"/>
       <c r="C2" s="140" t="inlineStr">
         <is>
-          <t>calculateSubtotal &amp; calculateDiscount</t>
+          <t>calculateSubtotal &amp; calculateDiscount &amp; calculateShippingFee</t>
         </is>
       </c>
       <c r="D2" s="139" t="n"/>
@@ -2861,7 +2861,7 @@
       <c r="K2" s="142" t="n"/>
       <c r="L2" s="143" t="inlineStr">
         <is>
-          <t>Tính thành tiền &amp; Chiết khấu</t>
+          <t>Tính thành tiền, Chiết khấu &amp; Phí giao hàng</t>
         </is>
       </c>
       <c r="M2" s="139" t="n"/>
@@ -2919,7 +2919,7 @@
       </c>
       <c r="B4" s="146" t="n"/>
       <c r="C4" s="107" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="D4" s="153" t="n"/>
       <c r="E4" s="7" t="n"/>
@@ -2954,7 +2954,7 @@
       <c r="B5" s="146" t="n"/>
       <c r="C5" s="115" t="inlineStr">
         <is>
-          <t>Kiểm thử đơn vị cho calculateSubtotal &amp; calculateDiscount (6 boundary values)</t>
+          <t>Kiểm thử đơn vị cho calculateSubtotal, calculateDiscount &amp; calculateShippingFee</t>
         </is>
       </c>
       <c r="D5" s="153" t="n"/>
@@ -3019,7 +3019,7 @@
     </row>
     <row r="7" ht="13.5" customHeight="1" thickBot="1">
       <c r="A7" s="162" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B7" s="163" t="n"/>
       <c r="C7" s="164" t="n">
@@ -3047,7 +3047,7 @@
         <v/>
       </c>
       <c r="O7" s="168" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="P7" s="165" t="n"/>
       <c r="Q7" s="165" t="n"/>
@@ -3108,9 +3108,21 @@
           <t>UTCID09</t>
         </is>
       </c>
-      <c r="O9" s="38" t="n"/>
-      <c r="P9" s="38" t="n"/>
-      <c r="Q9" s="38" t="n"/>
+      <c r="O9" s="38" t="inlineStr">
+        <is>
+          <t>UTCID10</t>
+        </is>
+      </c>
+      <c r="P9" s="38" t="inlineStr">
+        <is>
+          <t>UTCID11</t>
+        </is>
+      </c>
+      <c r="Q9" s="38" t="inlineStr">
+        <is>
+          <t>UTCID12</t>
+        </is>
+      </c>
       <c r="R9" s="38" t="n"/>
       <c r="S9" s="38" t="n"/>
       <c r="T9" s="39" t="n"/>
@@ -3272,9 +3284,21 @@
           <t>subtotal = 10000.0</t>
         </is>
       </c>
-      <c r="O13" s="11" t="n"/>
-      <c r="P13" s="11" t="n"/>
-      <c r="Q13" s="11" t="n"/>
+      <c r="O13" s="11" t="inlineStr">
+        <is>
+          <t>subtotal = 1999.99</t>
+        </is>
+      </c>
+      <c r="P13" s="11" t="inlineStr">
+        <is>
+          <t>subtotal = 2000.0</t>
+        </is>
+      </c>
+      <c r="Q13" s="11" t="inlineStr">
+        <is>
+          <t>subtotal = 5000.0</t>
+        </is>
+      </c>
       <c r="R13" s="11" t="n"/>
       <c r="S13" s="11" t="n"/>
       <c r="T13" s="28" t="n"/>
@@ -3885,9 +3909,21 @@
           <t>1500.0</t>
         </is>
       </c>
-      <c r="O38" s="46" t="n"/>
-      <c r="P38" s="46" t="n"/>
-      <c r="Q38" s="46" t="n"/>
+      <c r="O38" s="46" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="P38" s="46" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="Q38" s="46" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
       <c r="R38" s="46" t="n"/>
       <c r="S38" s="46" t="n"/>
       <c r="T38" s="47" t="n"/>
@@ -4139,9 +4175,21 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O47" s="82" t="n"/>
-      <c r="P47" s="82" t="n"/>
-      <c r="Q47" s="82" t="n"/>
+      <c r="O47" s="82" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="P47" s="82" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="Q47" s="82" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="R47" s="82" t="n"/>
       <c r="S47" s="82" t="n"/>
       <c r="T47" s="83" t="n"/>
@@ -4201,9 +4249,21 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="O48" s="19" t="n"/>
-      <c r="P48" s="19" t="n"/>
-      <c r="Q48" s="19" t="n"/>
+      <c r="O48" s="19" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="P48" s="19" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="Q48" s="19" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
       <c r="R48" s="19" t="n"/>
       <c r="S48" s="19" t="n"/>
       <c r="T48" s="84" t="n"/>
@@ -4263,9 +4323,21 @@
           <t>2026-10-04</t>
         </is>
       </c>
-      <c r="O49" s="173" t="n"/>
-      <c r="P49" s="173" t="n"/>
-      <c r="Q49" s="173" t="n"/>
+      <c r="O49" s="173" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="P49" s="173" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="Q49" s="173" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
       <c r="R49" s="173" t="n"/>
       <c r="S49" s="173" t="n"/>
       <c r="T49" s="84" t="n"/>
@@ -4325,9 +4397,21 @@
           <t>None</t>
         </is>
       </c>
-      <c r="O50" s="32" t="n"/>
-      <c r="P50" s="32" t="n"/>
-      <c r="Q50" s="32" t="n"/>
+      <c r="O50" s="32" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="P50" s="32" t="inlineStr">
+        <is>
+          <t>B03 (Fixed)</t>
+        </is>
+      </c>
+      <c r="Q50" s="32" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="R50" s="32" t="n"/>
       <c r="S50" s="32" t="n"/>
       <c r="T50" s="77" t="n"/>

</xml_diff>

<commit_message>
Fix bug B04 in calculateTotal correctly and pass all tests
</commit_message>
<xml_diff>
--- a/Unit_Test_Report.xlsx
+++ b/Unit_Test_Report.xlsx
@@ -2844,7 +2844,7 @@
       <c r="B2" s="139" t="n"/>
       <c r="C2" s="140" t="inlineStr">
         <is>
-          <t>calculateSubtotal &amp; calculateDiscount &amp; calculateShippingFee</t>
+          <t>calculateSubtotal &amp; calculateDiscount &amp; calculateShippingFee &amp; calculateTotal</t>
         </is>
       </c>
       <c r="D2" s="139" t="n"/>
@@ -2861,7 +2861,7 @@
       <c r="K2" s="142" t="n"/>
       <c r="L2" s="143" t="inlineStr">
         <is>
-          <t>Tính thành tiền, Chiết khấu &amp; Phí giao hàng</t>
+          <t>Tính tổng thanh toán đơn hàng</t>
         </is>
       </c>
       <c r="M2" s="139" t="n"/>
@@ -2919,7 +2919,7 @@
       </c>
       <c r="B4" s="146" t="n"/>
       <c r="C4" s="107" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="D4" s="153" t="n"/>
       <c r="E4" s="7" t="n"/>
@@ -2954,7 +2954,7 @@
       <c r="B5" s="146" t="n"/>
       <c r="C5" s="115" t="inlineStr">
         <is>
-          <t>Kiểm thử đơn vị cho calculateSubtotal, calculateDiscount &amp; calculateShippingFee</t>
+          <t>Kiểm thử đơn vị cho calculateSubtotal, calculateDiscount, calculateShippingFee &amp; calculateTotal</t>
         </is>
       </c>
       <c r="D5" s="153" t="n"/>
@@ -3019,7 +3019,7 @@
     </row>
     <row r="7" ht="13.5" customHeight="1" thickBot="1">
       <c r="A7" s="162" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B7" s="163" t="n"/>
       <c r="C7" s="164" t="n">
@@ -3047,7 +3047,7 @@
         <v/>
       </c>
       <c r="O7" s="168" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="P7" s="165" t="n"/>
       <c r="Q7" s="165" t="n"/>
@@ -3123,8 +3123,16 @@
           <t>UTCID12</t>
         </is>
       </c>
-      <c r="R9" s="38" t="n"/>
-      <c r="S9" s="38" t="n"/>
+      <c r="R9" s="38" t="inlineStr">
+        <is>
+          <t>UTCID13</t>
+        </is>
+      </c>
+      <c r="S9" s="38" t="inlineStr">
+        <is>
+          <t>UTCID14</t>
+        </is>
+      </c>
       <c r="T9" s="39" t="n"/>
       <c r="U9" s="27" t="n"/>
       <c r="V9" s="53" t="n"/>
@@ -3299,8 +3307,16 @@
           <t>subtotal = 5000.0</t>
         </is>
       </c>
-      <c r="R13" s="11" t="n"/>
-      <c r="S13" s="11" t="n"/>
+      <c r="R13" s="11" t="inlineStr">
+        <is>
+          <t>Product(price=500.0, qty=2)</t>
+        </is>
+      </c>
+      <c r="S13" s="11" t="inlineStr">
+        <is>
+          <t>Product(price=3000.0, qty=2)</t>
+        </is>
+      </c>
       <c r="T13" s="28" t="n"/>
       <c r="W13" s="58" t="n"/>
       <c r="X13" s="58" t="n"/>
@@ -3924,8 +3940,16 @@
           <t>0.0</t>
         </is>
       </c>
-      <c r="R38" s="46" t="n"/>
-      <c r="S38" s="46" t="n"/>
+      <c r="R38" s="46" t="inlineStr">
+        <is>
+          <t>1000.0</t>
+        </is>
+      </c>
+      <c r="S38" s="46" t="inlineStr">
+        <is>
+          <t>5400.0</t>
+        </is>
+      </c>
       <c r="T38" s="47" t="n"/>
     </row>
     <row r="39" ht="13.5" customHeight="1">
@@ -4190,8 +4214,16 @@
           <t>N</t>
         </is>
       </c>
-      <c r="R47" s="82" t="n"/>
-      <c r="S47" s="82" t="n"/>
+      <c r="R47" s="82" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S47" s="82" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="T47" s="83" t="n"/>
     </row>
     <row r="48">
@@ -4264,8 +4296,16 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="R48" s="19" t="n"/>
-      <c r="S48" s="19" t="n"/>
+      <c r="R48" s="19" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="S48" s="19" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
       <c r="T48" s="84" t="n"/>
     </row>
     <row r="49">
@@ -4338,8 +4378,16 @@
           <t>2026-10-04</t>
         </is>
       </c>
-      <c r="R49" s="173" t="n"/>
-      <c r="S49" s="173" t="n"/>
+      <c r="R49" s="173" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="S49" s="173" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
       <c r="T49" s="84" t="n"/>
     </row>
     <row r="50" ht="10.8" customHeight="1" thickBot="1">
@@ -4412,8 +4460,16 @@
           <t>None</t>
         </is>
       </c>
-      <c r="R50" s="32" t="n"/>
-      <c r="S50" s="32" t="n"/>
+      <c r="R50" s="32" t="inlineStr">
+        <is>
+          <t>B04 (Fixed)</t>
+        </is>
+      </c>
+      <c r="S50" s="32" t="inlineStr">
+        <is>
+          <t>B04 (Fixed)</t>
+        </is>
+      </c>
       <c r="T50" s="77" t="n"/>
     </row>
     <row r="51">

</xml_diff>

<commit_message>
Fix bug B05 in classifyCustomer and pass all tests
</commit_message>
<xml_diff>
--- a/Unit_Test_Report.xlsx
+++ b/Unit_Test_Report.xlsx
@@ -2844,7 +2844,7 @@
       <c r="B2" s="139" t="n"/>
       <c r="C2" s="140" t="inlineStr">
         <is>
-          <t>calculateSubtotal &amp; calculateDiscount &amp; calculateShippingFee &amp; calculateTotal</t>
+          <t>calculateSubtotal, calculateDiscount, calculateShippingFee, calculateTotal, classifyCustomer</t>
         </is>
       </c>
       <c r="D2" s="139" t="n"/>
@@ -2861,7 +2861,7 @@
       <c r="K2" s="142" t="n"/>
       <c r="L2" s="143" t="inlineStr">
         <is>
-          <t>Tính tổng thanh toán đơn hàng</t>
+          <t>Phân loại khách hàng</t>
         </is>
       </c>
       <c r="M2" s="139" t="n"/>
@@ -2919,7 +2919,7 @@
       </c>
       <c r="B4" s="146" t="n"/>
       <c r="C4" s="107" t="n">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="D4" s="153" t="n"/>
       <c r="E4" s="7" t="n"/>
@@ -2954,7 +2954,7 @@
       <c r="B5" s="146" t="n"/>
       <c r="C5" s="115" t="inlineStr">
         <is>
-          <t>Kiểm thử đơn vị cho calculateSubtotal, calculateDiscount, calculateShippingFee &amp; calculateTotal</t>
+          <t>Kiểm thử đơn vị đầy đủ 5 phương thức trong SalesService</t>
         </is>
       </c>
       <c r="D5" s="153" t="n"/>
@@ -3019,7 +3019,7 @@
     </row>
     <row r="7" ht="13.5" customHeight="1" thickBot="1">
       <c r="A7" s="162" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B7" s="163" t="n"/>
       <c r="C7" s="164" t="n">
@@ -3047,7 +3047,7 @@
         <v/>
       </c>
       <c r="O7" s="168" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="P7" s="165" t="n"/>
       <c r="Q7" s="165" t="n"/>
@@ -3133,9 +3133,26 @@
           <t>UTCID14</t>
         </is>
       </c>
-      <c r="T9" s="39" t="n"/>
-      <c r="U9" s="27" t="n"/>
-      <c r="V9" s="53" t="n"/>
+      <c r="T9" s="39" t="inlineStr">
+        <is>
+          <t>UTCID15</t>
+        </is>
+      </c>
+      <c r="U9" s="27" t="inlineStr">
+        <is>
+          <t>UTCID16</t>
+        </is>
+      </c>
+      <c r="V9" s="53" t="inlineStr">
+        <is>
+          <t>UTCID17</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>UTCID18</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="13.5" customHeight="1">
       <c r="A10" s="35" t="inlineStr">
@@ -3317,8 +3334,26 @@
           <t>Product(price=3000.0, qty=2)</t>
         </is>
       </c>
-      <c r="T13" s="28" t="n"/>
-      <c r="W13" s="58" t="n"/>
+      <c r="T13" s="28" t="inlineStr">
+        <is>
+          <t>total = 999.99</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>total = 1000.0</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>total = 5000.0</t>
+        </is>
+      </c>
+      <c r="W13" s="58" t="inlineStr">
+        <is>
+          <t>total = 10000.0</t>
+        </is>
+      </c>
       <c r="X13" s="58" t="n"/>
       <c r="Y13" s="58" t="n"/>
       <c r="Z13" s="58" t="n"/>
@@ -3950,7 +3985,26 @@
           <t>5400.0</t>
         </is>
       </c>
-      <c r="T38" s="47" t="n"/>
+      <c r="T38" s="47" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>SILVER</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>VIP</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="13.5" customHeight="1">
       <c r="A39" s="72" t="n"/>
@@ -4224,7 +4278,26 @@
           <t>N</t>
         </is>
       </c>
-      <c r="T47" s="83" t="n"/>
+      <c r="T47" s="83" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="72" t="n"/>
@@ -4306,7 +4379,26 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="T48" s="84" t="n"/>
+      <c r="T48" s="84" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="72" t="n"/>
@@ -4388,7 +4480,26 @@
           <t>2026-10-04</t>
         </is>
       </c>
-      <c r="T49" s="84" t="n"/>
+      <c r="T49" s="84" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="W49" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="10.8" customHeight="1" thickBot="1">
       <c r="A50" s="73" t="n"/>
@@ -4470,7 +4581,26 @@
           <t>B04 (Fixed)</t>
         </is>
       </c>
-      <c r="T50" s="77" t="n"/>
+      <c r="T50" s="77" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>B05 (Fixed)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="22" t="n"/>

</xml_diff>